<commit_message>
Month wise target changed
</commit_message>
<xml_diff>
--- a/2026-27_Year data_repots.xlsx
+++ b/2026-27_Year data_repots.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ack\My Drive\HINDUPUR-2022-2025\Target 2026-2027\report testing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ack\OneDrive\Documents\enforcement report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74DA515C-8820-462A-A549-F503DE140BA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888E6C84-D33C-4DF6-9973-D1D01953B5F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>